<commit_message>
full_rack_testplan.xlsx: TC-BMC-001..006 rows (BMC over Redfish, read-only; added 20 Oct 2026)
Scope 'BMC (Switch + Compute)', Origin 'Added - helios-tests (20 Oct 2026)', Non-disruptive, not run yet; appended
after row 583 with the look of the other added rows, filter range extended. The Execution Summary counts
(rows 3-1000) need no change; Excel recalculates their cached values on the next open.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testplan/full_rack_testplan.xlsx
+++ b/testplan/full_rack_testplan.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Execution Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Testcases'!$A$2:$L$583</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Testcases'!$A$2:$L$589</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -5235,7 +5235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M583"/>
+  <dimension ref="A1:M589"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="5" min="1" max="1"/>
@@ -36745,8 +36745,320 @@
         </is>
       </c>
     </row>
+    <row r="584" ht="32" customHeight="1" s="33">
+      <c r="A584" s="7" t="inlineStr">
+        <is>
+          <t>TC-BMC-001</t>
+        </is>
+      </c>
+      <c r="B584" s="7" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C584" s="5" t="inlineStr">
+        <is>
+          <t>BMC reachable and login works: every switch and compute BMC answers Redfish at its own address (bmc:) with its bmc_user and BMC password</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H584" s="21" t="inlineStr">
+        <is>
+          <t>Not run yet: added 20 Oct 2026, automated (tests/bmc/test_bmc.py, read-only Redfish); needs each node's bmc / bmc_user in the inventory and a BMC password (UI: Inventory tab default or Setup node table)</t>
+        </is>
+      </c>
+      <c r="I584" s="21" t="inlineStr">
+        <is>
+          <t>BMC Redfish (HTTPS) from the test runner</t>
+        </is>
+      </c>
+      <c r="J584" s="21" t="inlineStr">
+        <is>
+          <t>BMC (Switch + Compute)</t>
+        </is>
+      </c>
+      <c r="K584" s="21" t="inlineStr">
+        <is>
+          <t>Added - helios-tests (20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="L584" s="21" t="inlineStr">
+        <is>
+          <t>Non-disruptive</t>
+        </is>
+      </c>
+    </row>
+    <row r="585" ht="32" customHeight="1" s="33">
+      <c r="A585" s="7" t="inlineStr">
+        <is>
+          <t>TC-BMC-002</t>
+        </is>
+      </c>
+      <c r="B585" s="7" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C585" s="5" t="inlineStr">
+        <is>
+          <t>BMC power state: every system the switch and compute BMCs report is powered on</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H585" s="21" t="inlineStr">
+        <is>
+          <t>Not run yet: added 20 Oct 2026, automated (tests/bmc/test_bmc.py, read-only Redfish); needs each node's bmc / bmc_user in the inventory and a BMC password (UI: Inventory tab default or Setup node table)</t>
+        </is>
+      </c>
+      <c r="I585" s="21" t="inlineStr">
+        <is>
+          <t>BMC Redfish (HTTPS) from the test runner</t>
+        </is>
+      </c>
+      <c r="J585" s="21" t="inlineStr">
+        <is>
+          <t>BMC (Switch + Compute)</t>
+        </is>
+      </c>
+      <c r="K585" s="21" t="inlineStr">
+        <is>
+          <t>Added - helios-tests (20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="L585" s="21" t="inlineStr">
+        <is>
+          <t>Non-disruptive</t>
+        </is>
+      </c>
+    </row>
+    <row r="586" ht="32" customHeight="1" s="33">
+      <c r="A586" s="7" t="inlineStr">
+        <is>
+          <t>TC-BMC-003</t>
+        </is>
+      </c>
+      <c r="B586" s="7" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C586" s="5" t="inlineStr">
+        <is>
+          <t>BMC health: no BMC (manager) or system reports health Critical (Warning recorded)</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H586" s="21" t="inlineStr">
+        <is>
+          <t>Not run yet: added 20 Oct 2026, automated (tests/bmc/test_bmc.py, read-only Redfish); needs each node's bmc / bmc_user in the inventory and a BMC password (UI: Inventory tab default or Setup node table)</t>
+        </is>
+      </c>
+      <c r="I586" s="21" t="inlineStr">
+        <is>
+          <t>BMC Redfish (HTTPS) from the test runner</t>
+        </is>
+      </c>
+      <c r="J586" s="21" t="inlineStr">
+        <is>
+          <t>BMC (Switch + Compute)</t>
+        </is>
+      </c>
+      <c r="K586" s="21" t="inlineStr">
+        <is>
+          <t>Added - helios-tests (20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="L586" s="21" t="inlineStr">
+        <is>
+          <t>Non-disruptive</t>
+        </is>
+      </c>
+    </row>
+    <row r="587" ht="32" customHeight="1" s="33">
+      <c r="A587" s="7" t="inlineStr">
+        <is>
+          <t>TC-BMC-004</t>
+        </is>
+      </c>
+      <c r="B587" s="7" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C587" s="5" t="inlineStr">
+        <is>
+          <t>BMC sensors: no temperature, fan, voltage or power-supply sensor Critical or beyond its critical limit (beyond a non-critical limit recorded)</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H587" s="21" t="inlineStr">
+        <is>
+          <t>Not run yet: added 20 Oct 2026, automated (tests/bmc/test_bmc.py, read-only Redfish); needs each node's bmc / bmc_user in the inventory and a BMC password (UI: Inventory tab default or Setup node table)</t>
+        </is>
+      </c>
+      <c r="I587" s="21" t="inlineStr">
+        <is>
+          <t>BMC Redfish (HTTPS) from the test runner</t>
+        </is>
+      </c>
+      <c r="J587" s="21" t="inlineStr">
+        <is>
+          <t>BMC (Switch + Compute)</t>
+        </is>
+      </c>
+      <c r="K587" s="21" t="inlineStr">
+        <is>
+          <t>Added - helios-tests (20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="L587" s="21" t="inlineStr">
+        <is>
+          <t>Non-disruptive</t>
+        </is>
+      </c>
+    </row>
+    <row r="588" ht="32" customHeight="1" s="33">
+      <c r="A588" s="7" t="inlineStr">
+        <is>
+          <t>TC-BMC-005</t>
+        </is>
+      </c>
+      <c r="B588" s="7" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C588" s="5" t="inlineStr">
+        <is>
+          <t>BMC event log: no Critical entry in the last 24 h (thresholds.bmc.log_window_h); Warning entries counted</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H588" s="21" t="inlineStr">
+        <is>
+          <t>Not run yet: added 20 Oct 2026, automated (tests/bmc/test_bmc.py, read-only Redfish); needs each node's bmc / bmc_user in the inventory and a BMC password (UI: Inventory tab default or Setup node table)</t>
+        </is>
+      </c>
+      <c r="I588" s="21" t="inlineStr">
+        <is>
+          <t>BMC Redfish (HTTPS) from the test runner</t>
+        </is>
+      </c>
+      <c r="J588" s="21" t="inlineStr">
+        <is>
+          <t>BMC (Switch + Compute)</t>
+        </is>
+      </c>
+      <c r="K588" s="21" t="inlineStr">
+        <is>
+          <t>Added - helios-tests (20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="L588" s="21" t="inlineStr">
+        <is>
+          <t>Non-disruptive</t>
+        </is>
+      </c>
+    </row>
+    <row r="589" ht="32" customHeight="1" s="33">
+      <c r="A589" s="7" t="inlineStr">
+        <is>
+          <t>TC-BMC-006</t>
+        </is>
+      </c>
+      <c r="B589" s="7" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C589" s="5" t="inlineStr">
+        <is>
+          <t>BMC firmware consistent: same BMC firmware version on every compute tray, and on every switch tray</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H589" s="21" t="inlineStr">
+        <is>
+          <t>Not run yet: added 20 Oct 2026, automated (tests/bmc/test_bmc.py, read-only Redfish); needs each node's bmc / bmc_user in the inventory and a BMC password (UI: Inventory tab default or Setup node table)</t>
+        </is>
+      </c>
+      <c r="I589" s="21" t="inlineStr">
+        <is>
+          <t>BMC Redfish (HTTPS) from the test runner</t>
+        </is>
+      </c>
+      <c r="J589" s="21" t="inlineStr">
+        <is>
+          <t>BMC (Switch + Compute)</t>
+        </is>
+      </c>
+      <c r="K589" s="21" t="inlineStr">
+        <is>
+          <t>Added - helios-tests (20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="L589" s="21" t="inlineStr">
+        <is>
+          <t>Non-disruptive</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L583">
+  <autoFilter ref="A2:L589">
     <filterColumn colId="3" hiddenButton="0" showButton="1">
       <filters>
         <filter val="No"/>

</xml_diff>

<commit_message>
Test plan: TC-AFM-005A / TC-AFM-048A get their own IDs (were shared with TC-AFM-005 / 048)
- full_rack_testplan.xlsx: row 7 (RCCL Cross Domain) TC-AFM-005 -> TC-AFM-005A, row 52 (Audit Events) TC-AFM-048 ->
  TC-AFM-048A - the IDs their automated tests already used; a dated note on each row says what it was in the
  BKC-26.12 plan. No duplicate IDs left (696 rows, 696 IDs).
- update_testplan.find_row: a case's own ID first (a once-shared one must still match its title), else the old shared
  TID + title of ROW_ALIASES, so older workbook copies keep working. unit/test_testplan_rows covers both layouts.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testplan/full_rack_testplan.xlsx
+++ b/testplan/full_rack_testplan.xlsx
@@ -5580,7 +5580,7 @@
     <row r="7" hidden="1" ht="32" customHeight="1" s="33">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>TC-AFM-005</t>
+          <t>TC-AFM-005A</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -5610,7 +5610,8 @@
       </c>
       <c r="H7" s="21" t="inlineStr">
         <is>
-          <t>[g02-g17 full rack, 16 Oct 13:48 UTC, helios-tests g02-g17-20261016-135436] Pending: rccl-tests not installed on any tray and no cross-domain launch configured; AMD reports the cross-domain RCCL smoke test passing - asked for their command.
+          <t>[ID renamed 21 Oct 2026] TC-AFM-005 in the BKC-26.12 plan, where it was shared with 'Failover Policy CRUD' - renumbered TC-AFM-005A, the ID its automated test already used.
+Earlier: [g02-g17 full rack, 16 Oct 13:48 UTC, helios-tests g02-g17-20261016-135436] Pending: rccl-tests not installed on any tray and no cross-domain launch configured; AMD reports the cross-domain RCCL smoke test passing - asked for their command.
 Earlier: [g02-g17 full rack, L1 rerun with sudo, 14 Oct 2026 15:11-15:35 UTC, helios-tests g02-g17-20261014-153550] Pending: rccl-tests not installed / no cross-domain launch configured. Evidence: RcclSmokeTest multi-node failed because CT15 could not open its GPUs (the other ranks were stopped at once). Pre-flight excluded: CT02/CT05 down (no SSH, BMC up); CT01 GPUs in use by another team's job (/user/hpe/dtm/mlperf-poc ... gpu-flops).
 Earlier: [g02-g17 full rack, L1, 14 Oct 2026, helios-tests g02-g17-20261014-143740 + pre-flight 134911] Not run: rccl-tests not installed and commands.rccl.cross_domain not set. Evidence RcclSmokeTest multi-node FAILED: 'invalid argument' (ranks on CT01) and 'no ROCm-capable device' (CT03+), same GPU permission cause. Run 13:49-14:37 UTC from the jump host on 15 trays: CT02/CT05 down (no ping, BMC up); CT18 excluded (black-holed ports, see TC-AFM-001). Root cause of the GPU errors: the test account tenant-hpe is not in the 'render' group, so it cannot open /dev/kfd (amd-smi: permission denied) - rerun with sudo (commands.datapath.sudo) or after adding the account to 'render'. Another HPE workload (palsd, /var/tmp/HPE sc framework) was also running.
 Earlier: 12 Oct traffic validation T4: RcclSmokeTest across 18 trays / 72 ranks from CT01; 21/21 cells incl. 1 GB, all processes exited cleanly, exit 0.</t>
@@ -8132,7 +8133,7 @@
     <row r="52" hidden="1" ht="16" customHeight="1" s="33">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>TC-AFM-048</t>
+          <t>TC-AFM-048A</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -8162,7 +8163,8 @@
       </c>
       <c r="H52" s="21" t="inlineStr">
         <is>
-          <t>[g02-g17 full rack, non-disruptive switch + AFM API, 14 Oct 2026] 1 item(s) passed (helios-tests fullrack-switch-nd-filtered, g02-g17-20261014-092828, g02-g17-20261014-170350, g02-g17-20261014-170910)
+          <t>[ID renamed 21 Oct 2026] TC-AFM-048 in the BKC-26.12 plan, where it was shared with 'Techsupport Validation (Sideband Only)' - renumbered TC-AFM-048A, the ID its automated test already used.
+Earlier: [g02-g17 full rack, non-disruptive switch + AFM API, 14 Oct 2026] 1 item(s) passed (helios-tests fullrack-switch-nd-filtered, g02-g17-20261014-092828, g02-g17-20261014-170350, g02-g17-20261014-170910)
 Earlier: CRUD + login audit events present; duplicate Delete/requestauthorization is a known WARN (AIFM-1363).</t>
         </is>
       </c>

</xml_diff>